<commit_message>
<finish the data analysis of questionair>
</commit_message>
<xml_diff>
--- a/MCM/2025/C/result/result_2028.xlsx
+++ b/MCM/2025/C/result/result_2028.xlsx
@@ -478,29 +478,29 @@
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D3" t="n">
-        <v>150</v>
+        <v>123</v>
       </c>
       <c r="E3" t="n">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="F3" t="n">
-        <v>424</v>
+        <v>415</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>0.6</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.61</v>
+        <v>0.55</v>
       </c>
       <c r="E4" t="n">
-        <v>0.61</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -534,13 +534,13 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>0.63</v>
+        <v>0.7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="E6" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -574,13 +574,13 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="D8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.87</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.85</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="D10" t="n">
         <v>0.91</v>
@@ -654,13 +654,13 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="D12" t="n">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="E12" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -694,13 +694,13 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>0.78</v>
+        <v>0.73</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -734,13 +734,13 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>0.82</v>
+        <v>0.78</v>
       </c>
       <c r="D16" t="n">
-        <v>0.89</v>
+        <v>0.85</v>
       </c>
       <c r="E16" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -774,13 +774,13 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="E18" t="n">
-        <v>0.67</v>
+        <v>0.75</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -814,13 +814,13 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>0.82</v>
+        <v>0.91</v>
       </c>
       <c r="D20" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.87</v>
       </c>
       <c r="E20" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -854,13 +854,13 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>0.91</v>
+        <v>0.85</v>
       </c>
       <c r="D22" t="n">
         <v>0.87</v>
       </c>
       <c r="E22" t="n">
-        <v>0.88</v>
+        <v>0.8</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -894,13 +894,13 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>0.65</v>
+        <v>0.63</v>
       </c>
       <c r="D24" t="n">
-        <v>0.68</v>
+        <v>0.62</v>
       </c>
       <c r="E24" t="n">
-        <v>0.62</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -934,13 +934,13 @@
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="D26" t="n">
-        <v>0.91</v>
+        <v>0.9</v>
       </c>
       <c r="E26" t="n">
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -974,13 +974,13 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>0.65</v>
+        <v>0.58</v>
       </c>
       <c r="D28" t="n">
-        <v>0.57</v>
+        <v>0.53</v>
       </c>
       <c r="E28" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1014,13 +1014,13 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="D30" t="n">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="E30" t="n">
-        <v>0.83</v>
+        <v>0.87</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1054,13 +1054,13 @@
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="D32" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.91</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1094,13 +1094,13 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E34" t="n">
         <v>0.53</v>
-      </c>
-      <c r="D34" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0.61</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1134,13 +1134,13 @@
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="D36" t="n">
         <v>0.7</v>
       </c>
-      <c r="D36" t="n">
-        <v>0.8</v>
-      </c>
       <c r="E36" t="n">
-        <v>0.63</v>
+        <v>0.7</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1174,13 +1174,13 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="D38" t="n">
-        <v>0.6</v>
+        <v>0.74</v>
       </c>
       <c r="E38" t="n">
-        <v>0.6</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="n">
-        <v>0.61</v>
+        <v>0.72</v>
       </c>
       <c r="D42" t="n">
         <v>0.88</v>
@@ -1296,13 +1296,13 @@
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E44" t="n">
         <v>0.7</v>
-      </c>
-      <c r="D44" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0.6</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1336,13 +1336,13 @@
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="D46" t="n">
-        <v>0.72</v>
+        <v>0.68</v>
       </c>
       <c r="E46" t="n">
-        <v>0.64</v>
+        <v>0.58</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -1376,10 +1376,10 @@
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="n">
-        <v>0.67</v>
+        <v>0.64</v>
       </c>
       <c r="D48" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1418,10 +1418,10 @@
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="D50" t="n">
-        <v>0.7</v>
+        <v>0.64</v>
       </c>
       <c r="E50" t="n">
         <v>0.77</v>
@@ -1458,13 +1458,13 @@
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D52" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="D52" t="n">
-        <v>0.9</v>
-      </c>
       <c r="E52" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -1498,13 +1498,13 @@
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="n">
-        <v>0.67</v>
+        <v>0.64</v>
       </c>
       <c r="D54" t="n">
-        <v>0.71</v>
+        <v>0.57</v>
       </c>
       <c r="E54" t="n">
-        <v>0.55</v>
+        <v>0.61</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -1538,7 +1538,7 @@
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="n">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.67</v>
+        <v>0.82</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -1580,13 +1580,13 @@
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="n">
-        <v>0.71</v>
+        <v>0.52</v>
       </c>
       <c r="D58" t="n">
-        <v>0.73</v>
+        <v>0.66</v>
       </c>
       <c r="E58" t="n">
-        <v>0.59</v>
+        <v>0.57</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -1620,13 +1620,13 @@
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="n">
-        <v>0.5</v>
+        <v>0.59</v>
       </c>
       <c r="D60" t="n">
-        <v>0.73</v>
+        <v>0.65</v>
       </c>
       <c r="E60" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -1660,13 +1660,13 @@
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="n">
-        <v>0.5</v>
+        <v>0.64</v>
       </c>
       <c r="D62" t="n">
-        <v>0.65</v>
+        <v>0.61</v>
       </c>
       <c r="E62" t="n">
-        <v>0.68</v>
+        <v>0.6</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -1700,13 +1700,13 @@
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="n">
-        <v>0.55</v>
+        <v>0.64</v>
       </c>
       <c r="D64" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="E64" t="n">
-        <v>0.63</v>
+        <v>0.75</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -1740,13 +1740,13 @@
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="D66" t="n">
-        <v>0.9</v>
+        <v>0.61</v>
       </c>
       <c r="E66" t="n">
-        <v>0.8</v>
+        <v>0.59</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -1780,10 +1780,10 @@
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="n">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="D68" t="n">
-        <v>0.7</v>
+        <v>0.64</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="n">
-        <v>0.85</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.65</v>
+        <v>0.87</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="n">
-        <v>0.78</v>
+        <v>0.59</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -1914,7 +1914,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -1992,13 +1992,13 @@
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="n">
-        <v>0.5</v>
+        <v>0.72</v>
       </c>
       <c r="D78" t="n">
-        <v>0.74</v>
+        <v>0.6</v>
       </c>
       <c r="E78" t="n">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -2032,13 +2032,13 @@
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="n">
-        <v>0.61</v>
+        <v>0.49</v>
       </c>
       <c r="D80" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.64</v>
       </c>
       <c r="E80" t="n">
-        <v>0.63</v>
+        <v>0.57</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -2072,13 +2072,13 @@
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="n">
-        <v>0.51</v>
+        <v>0.48</v>
       </c>
       <c r="D82" t="n">
-        <v>0.62</v>
+        <v>0.54</v>
       </c>
       <c r="E82" t="n">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -2112,13 +2112,13 @@
       <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="D84" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E84" t="n">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -2152,13 +2152,13 @@
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="n">
-        <v>0.6</v>
+        <v>0.54</v>
       </c>
       <c r="D86" t="n">
-        <v>0.55</v>
+        <v>0.57</v>
       </c>
       <c r="E86" t="n">
-        <v>0.6</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -2192,13 +2192,13 @@
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="n">
-        <v>0.5</v>
+        <v>0.68</v>
       </c>
       <c r="D88" t="n">
-        <v>0.7</v>
+        <v>0.64</v>
       </c>
       <c r="E88" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -2232,10 +2232,10 @@
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="n">
-        <v>0.62</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D90" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2274,13 +2274,13 @@
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="n">
-        <v>0.67</v>
+        <v>0.53</v>
       </c>
       <c r="D92" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="E92" t="n">
         <v>0.6</v>
-      </c>
-      <c r="E92" t="n">
-        <v>0.62</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -2314,13 +2314,13 @@
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D94" t="n">
-        <v>0.53</v>
+        <v>0.67</v>
       </c>
       <c r="E94" t="n">
-        <v>0.51</v>
+        <v>0.55</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="n">
-        <v>0.6</v>
+        <v>0.54</v>
       </c>
       <c r="D96" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="E96" t="n">
         <v>0.6</v>
@@ -2394,13 +2394,13 @@
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="n">
-        <v>0.78</v>
+        <v>0.58</v>
       </c>
       <c r="D98" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="E98" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -2434,10 +2434,10 @@
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="n">
-        <v>0.9</v>
+        <v>0.93</v>
       </c>
       <c r="D100" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E100" t="n">
         <v>0.87</v>
@@ -2474,13 +2474,13 @@
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="n">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="D102" t="n">
-        <v>0.8</v>
+        <v>0.66</v>
       </c>
       <c r="E102" t="n">
-        <v>0.66</v>
+        <v>0.72</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -2514,13 +2514,13 @@
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="n">
-        <v>0.58</v>
+        <v>0.53</v>
       </c>
       <c r="D104" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="E104" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.54</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -2554,13 +2554,13 @@
       <c r="A106" t="inlineStr"/>
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="n">
-        <v>0.6</v>
+        <v>0.57</v>
       </c>
       <c r="D106" t="n">
-        <v>0.8</v>
+        <v>0.62</v>
       </c>
       <c r="E106" t="n">
-        <v>0.8</v>
+        <v>0.57</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -2594,10 +2594,10 @@
       <c r="A108" t="inlineStr"/>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="n">
-        <v>0.7</v>
+        <v>0.62</v>
       </c>
       <c r="D108" t="n">
-        <v>0.8</v>
+        <v>0.59</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2636,10 +2636,10 @@
       <c r="A110" t="inlineStr"/>
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="n">
-        <v>0.62</v>
+        <v>0.51</v>
       </c>
       <c r="D110" t="n">
-        <v>0.7</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2678,10 +2678,10 @@
       <c r="A112" t="inlineStr"/>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="D112" t="n">
-        <v>0.5</v>
+        <v>0.64</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2720,10 +2720,10 @@
       <c r="A114" t="inlineStr"/>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="n">
-        <v>0.5</v>
+        <v>0.68</v>
       </c>
       <c r="D114" t="n">
-        <v>0.48</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2762,7 +2762,7 @@
       <c r="A116" t="inlineStr"/>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -2770,7 +2770,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>0.77</v>
+        <v>0.65</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -2804,7 +2804,7 @@
       <c r="A118" t="inlineStr"/>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="n">
-        <v>0.6</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>0.46</v>
+        <v>0.61</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -2846,7 +2846,7 @@
       <c r="A120" t="inlineStr"/>
       <c r="B120" t="inlineStr"/>
       <c r="C120" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -2854,7 +2854,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>0.9</v>
+        <v>0.62</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -2888,7 +2888,7 @@
       <c r="A122" t="inlineStr"/>
       <c r="B122" t="inlineStr"/>
       <c r="C122" t="n">
-        <v>0.9</v>
+        <v>0.62</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>0.5</v>
+        <v>0.46</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
       <c r="A124" t="inlineStr"/>
       <c r="B124" t="inlineStr"/>
       <c r="C124" t="n">
-        <v>0.52</v>
+        <v>0.55</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>1</v>
+        <v>0.55</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -2972,7 +2972,7 @@
       <c r="A126" t="inlineStr"/>
       <c r="B126" t="inlineStr"/>
       <c r="C126" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -3016,7 +3016,7 @@
       <c r="A128" t="inlineStr"/>
       <c r="B128" t="inlineStr"/>
       <c r="C128" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -3065,10 +3065,10 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>0.93</v>
+        <v>0.78</v>
       </c>
       <c r="E130" t="n">
-        <v>0.83</v>
+        <v>0.78</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -3107,10 +3107,10 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="E132" t="n">
-        <v>0.6</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.57</v>
+        <v>0.65</v>
       </c>
       <c r="E134" t="n">
-        <v>0.6</v>
+        <v>0.72</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -3191,10 +3191,10 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>0.6</v>
+        <v>0.53</v>
       </c>
       <c r="E136" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -3233,10 +3233,10 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="E138" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -3275,10 +3275,10 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="E140" t="n">
-        <v>0.65</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -3317,10 +3317,10 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="E142" t="n">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -3359,10 +3359,10 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>0.6</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E144" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="F144" t="inlineStr">
         <is>
@@ -3401,10 +3401,10 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0.51</v>
+        <v>0.45</v>
       </c>
       <c r="E146" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="F146" t="inlineStr">
         <is>
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.5</v>
+        <v>0.64</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.7</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -3575,7 +3575,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.5</v>
+        <v>0.65</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -3668,7 +3668,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>0.8</v>
+        <v>0.68</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -3712,7 +3712,7 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>0.55</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="F162" t="inlineStr">
         <is>
@@ -3800,7 +3800,7 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>0.75</v>
+        <v>0.61</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
@@ -3844,7 +3844,7 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>0.8</v>
+        <v>0.74</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
@@ -3888,7 +3888,7 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>0.7</v>
+        <v>0.59</v>
       </c>
       <c r="F168" t="inlineStr">
         <is>
@@ -3932,7 +3932,7 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>0.8</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F170" t="inlineStr">
         <is>
@@ -3976,7 +3976,7 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="F172" t="inlineStr">
         <is>
@@ -4020,7 +4020,7 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>0.7</v>
+        <v>0.59</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -4064,7 +4064,7 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>0.5</v>
+        <v>0.64</v>
       </c>
       <c r="F176" t="inlineStr">
         <is>

</xml_diff>